<commit_message>
docs(scale): harmonize 100 concurrent and 1000 daily meetings scale metrics across ITS-209 and ITS-237
</commit_message>
<xml_diff>
--- a/ITS-209-Technology-Plan-IV-Indexing.xlsx
+++ b/ITS-209-Technology-Plan-IV-Indexing.xlsx
@@ -886,7 +886,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Enterprise automated Microsoft Teams Calling Bot application (TDA Bot) that automatically attends enterprise Teams meetings, captures real-time unmixed audio and video feeds via Microsoft Graph Calling SDK and Skype Media Platform, transcribes speech with speaker diarization using OpenAI Whisper, and generates structured Minutes of Meeting (MoM) documents in Word (.docx) format delivered directly to meeting organizers. The system features in-call chat command interaction (@TDA #joinv2, #status, #stop, #leave), real-time mascot status video broadcasting, and centralized meeting archival to Google Cloud Storage and BigQuery.</t>
+          <t>Enterprise automated Microsoft Teams Calling Bot application (TDA Bot) engineered to scale up to 100 concurrent meetings and 1,000 daily meetings across Tata Steel. The bot automatically attends Teams meetings, captures real-time unmixed audio and video feeds via Microsoft Graph Calling SDK and Skype Media Platform, transcribes speech with speaker diarization using OpenAI Whisper, and generates structured Minutes of Meeting (MoM) documents in Word (.docx) format delivered directly to organizers. Features in-call chat controls (@TDA #joinv2, #status, #stop, #leave), real-time mascot status video broadcasting, and centralized meeting archival to Google Cloud Storage (GCS) and BigQuery.</t>
         </is>
       </c>
       <c r="D4" s="8" t="n"/>
@@ -998,7 +998,7 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>The solution integrates Microsoft Graph Calling SDK (.NET 4.7.2 x64 on Windows Media Platform VM) with Microsoft Teams tenant infrastructure. Azure Bot Service (Node.js) handles incoming chat commands and dispatches join requests. Real-time media sockets receive unmixed audio (PCM 16kHz) and video frames, which are recorded and processed by an automated Whisper transcription engine and LLM MoM generator. Final recordings, transcripts, and Word (.docx) MoM files are securely archived to Google Cloud Storage (GCS) with metadata and audit telemetry published to Google BigQuery. Concurrency and duplicate joins are coordinated via Google Cloud Firestore distributed locks.</t>
+          <t>The solution integrates Microsoft Graph Calling SDK (.NET 4.7.2 x64 on Windows Media Platform VM) with Microsoft Teams tenant infrastructure. Azure Bot Service (Node.js) handles incoming chat commands and dispatches join requests. Sized to process 100 concurrent meetings and 1,000 daily meetings. Real-time media sockets receive unmixed audio (PCM 16kHz) and video frames, which are recorded and processed by an automated Whisper transcription engine and LLM MoM generator. Final recordings, transcripts, and Word (.docx) MoM files are securely archived to Google Cloud Storage (GCS) with metadata and audit telemetry published to Google BigQuery. Concurrency and duplicate joins are coordinated via Google Cloud Firestore distributed locks.</t>
         </is>
       </c>
       <c r="D11" s="9" t="n"/>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Encrypted bucket storage for meeting recordings (.mp4/.wav), transcript JSONs, and Word (.docx) MoMs</t>
+          <t>Encrypted bucket storage for meeting recordings (.mp4/.wav), transcript JSONs, and Word (.docx) MoMs, sized for 1,000 daily meetings (~300-500 GB/day)</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Centralized meeting registry, transcript semantic search index, action item analytics, and audit logging</t>
+          <t>Centralized meeting registry, transcript semantic search index, action item analytics, and audit logging sized for 1,000 daily meetings (~30,000 meetings/month)</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>OpenAI Whisper (Large-v3/Medium) for speech-to-text &amp; Claude / Azure OpenAI LLM for MoM generation</t>
+          <t>OpenAI Whisper (Large-v3/Medium) &amp; Claude / Azure OpenAI LLM, sized to transcribe and summarize up to 100 concurrent meetings and 1,000 daily meetings</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Distributed call concurrency locks and real-time meeting state registry</t>
+          <t>Distributed call concurrency locks and real-time meeting state registry, coordinating 100 concurrent calls and 1,000 daily meetings without race conditions</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Requires dedicated Windows VM for Skype Media Platform native drivers &amp; real-time audio/video processing</t>
+          <t>Dedicated Windows VM cluster sized for 100 concurrent real-time audio/video streams and 1,000 daily meetings throughput with Skype Media Platform native drivers</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>250 GB NVMe/SSD transient media buffer (auto-purged post-upload)</t>
+          <t>250 GB NVMe/SSD transient media buffer (sized for 100 concurrent streams; auto-purged immediately upon GCS upload to support 1,000 daily meetings without disk overflow)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>10 GB (Meeting locks, active call states, participant registries)</t>
+          <t>10 GB (Serverless distributed concurrency locks &amp; call state registry, sized for 100 concurrent calls and 1,000 daily meetings / ~50k operations daily)</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>500 GB (Indexed transcripts, MoM summaries, attendee logs, call telemetry)</t>
+          <t>500 GB - 1 TB (Data warehouse sized for 1,000 daily meetings / ~30,000 monthly meetings; indexed transcripts, MoM summaries, attendee logs, call telemetry)</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Dedicated 1 Gbps NIC. Bandwidth consumption ~1.5 Mbps per concurrent audio/video meeting; supports 100 concurrent calls (~150-200 Mbps aggregate continuous throughput).</t>
+          <t>Dedicated 1 Gbps NIC. Bandwidth sized for 100 concurrent calls @ ~1.5 Mbps per call (~150-200 Mbps aggregate continuous throughput). Daily data transfer sized for 1,000 meetings per day (~300-500 GB daily media egress to Google Cloud Storage over enterprise 1 Gbps pipe).</t>
         </is>
       </c>
     </row>

</xml_diff>